<commit_message>
Actualizar la configuración compilada y los archivos de datos de Excel
</commit_message>
<xml_diff>
--- a/data/empleados.xlsx
+++ b/data/empleados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Bibliotecas\Documents\GitHub\TPI-Organizacion-empresarial\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24D8D9FB-0126-4D30-B995-0E54A32B89A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E31A9D5-3E2F-46F0-8882-999B89D5AF6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>DNI</t>
   </si>
@@ -55,6 +55,9 @@
   </si>
   <si>
     <t>Carolina Gregoris</t>
+  </si>
+  <si>
+    <t>Marcelo Berton</t>
   </si>
 </sst>
 </file>
@@ -382,7 +385,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.44140625" customWidth="1"/>
@@ -478,6 +481,17 @@
         <v>7</v>
       </c>
     </row>
+    <row r="9" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
+        <v>43438273</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" s="1">
+        <v>21</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>

</xml_diff>